<commit_message>
I file di prova hanno di nuovo la forma dei file veri
Erano rimasti alle colonne di prima: intestazione "Modello" invece di
"Modello/Descrizione", ordine vecchio, larghezze fisse. Un collaudo su
file che non somigliano piu' a quelli veri verifica una cosa che non
esiste.

Il generatore ora ricava colonne e ordine dal modello da compilare
invece di riscriverli, e una suite lega le due cose: se il modello
cambia e i file di prova restano indietro, il test cade.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Collaudo/Inventario_di_prova.xlsx
+++ b/Collaudo/Inventario_di_prova.xlsx
@@ -438,12 +438,12 @@
   <dimension ref="A1:F34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="36" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="27" customWidth="1" min="3" max="3"/>
+    <col width="25" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -459,22 +459,22 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Modello</t>
+          <t>Stato</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Modello/Descrizione</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>Numero di serie</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Stato</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Note</t>
         </is>
       </c>
     </row>
@@ -498,20 +498,20 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
+          <t>Disponibile</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
           <t>Lenovo ThinkPad T14 Gen 5</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>PF5BA01</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Disponibile</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -526,22 +526,22 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
+          <t>Disponibile</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Postazione 1</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
           <t>Lenovo ThinkPad T14 Gen 4</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>PF4BA02</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Disponibile</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Postazione 1</t>
         </is>
       </c>
     </row>
@@ -558,20 +558,20 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
+          <t>Disponibile</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
           <t>Lenovo ThinkPad T14 Gen 5</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>PF5BA03</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Disponibile</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -586,22 +586,22 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
+          <t>In attesa ritiro</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Batteria da sostituire</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
           <t>Lenovo ThinkPad T14 Gen 4</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>PF4BA04</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>In attesa ritiro</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Batteria da sostituire</t>
         </is>
       </c>
     </row>
@@ -618,20 +618,20 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
+          <t>Guasto in attesa tecnico</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
           <t>Lenovo ThinkPad T14 Gen 5</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>PF5BA05</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Guasto in attesa tecnico</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -646,22 +646,22 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
+          <t>Da rebuildare</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Con custodia</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
           <t>Lenovo ThinkPad T14 Gen 4</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>PF4BA06</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>Da rebuildare</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>Con custodia</t>
         </is>
       </c>
     </row>
@@ -678,20 +678,20 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
+          <t>Controllare</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr">
+        <is>
           <t>Lenovo ThinkPad T14 Gen 5</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="F9" t="inlineStr">
         <is>
           <t>PF5BA07</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>Controllare</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -706,22 +706,22 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
+          <t>Disponibile</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>In verifica</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
           <t>Dell Latitude 7320 Detachable</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t>7HB108</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>Disponibile</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>In verifica</t>
         </is>
       </c>
     </row>
@@ -738,20 +738,20 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
+          <t>Disponibile</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr">
+        <is>
           <t>Dell Latitude 7230 Rugged Extreme</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="F11" t="inlineStr">
         <is>
           <t>8HB109</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>Disponibile</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -766,22 +766,22 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
+          <t>Disponibile</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Scorta</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
           <t>Dell Latitude 7320 Detachable</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="F12" t="inlineStr">
         <is>
           <t>4HB110</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>Disponibile</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>Scorta</t>
         </is>
       </c>
     </row>
@@ -805,20 +805,20 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
+          <t>Disponibile</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr">
+        <is>
           <t>Lenovo ThinkPad T14 Gen 5</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="F14" t="inlineStr">
         <is>
           <t>PF5KS01</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>Disponibile</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -833,22 +833,22 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
+          <t>Disponibile</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Postazione 1</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
           <t>Lenovo ThinkPad T14 Gen 4</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="F15" t="inlineStr">
         <is>
           <t>PF4KS02</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>Disponibile</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>Postazione 1</t>
         </is>
       </c>
     </row>
@@ -865,20 +865,20 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
+          <t>Disponibile</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr">
+        <is>
           <t>Lenovo ThinkPad T14 Gen 5</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="F16" t="inlineStr">
         <is>
           <t>PF5KS03</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>Disponibile</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -893,22 +893,22 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
+          <t>In attesa ritiro</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Batteria da sostituire</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
           <t>Lenovo ThinkPad T14 Gen 4</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="F17" t="inlineStr">
         <is>
           <t>PF4KS04</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>In attesa ritiro</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>Batteria da sostituire</t>
         </is>
       </c>
     </row>
@@ -925,20 +925,20 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
+          <t>Guasto in attesa tecnico</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr">
+        <is>
           <t>Lenovo ThinkPad T14 Gen 5</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="F18" t="inlineStr">
         <is>
           <t>PF5KS05</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>Guasto in attesa tecnico</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -953,22 +953,22 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
+          <t>Da rebuildare</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Con custodia</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
           <t>Lenovo ThinkPad T14 Gen 4</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="F19" t="inlineStr">
         <is>
           <t>PF4KS06</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>Da rebuildare</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>Con custodia</t>
         </is>
       </c>
     </row>
@@ -985,20 +985,20 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
+          <t>Controllare</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr">
+        <is>
           <t>Lenovo ThinkPad T14 Gen 5</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="F20" t="inlineStr">
         <is>
           <t>PF5KS07</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>Controllare</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1013,22 +1013,22 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
+          <t>Disponibile</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>In verifica</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
           <t>Dell Latitude 7320 Detachable</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="F21" t="inlineStr">
         <is>
           <t>7HK208</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>Disponibile</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>In verifica</t>
         </is>
       </c>
     </row>
@@ -1045,20 +1045,20 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
+          <t>Disponibile</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr">
+        <is>
           <t>Dell Latitude 7230 Rugged Extreme</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="F22" t="inlineStr">
         <is>
           <t>8HK209</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>Disponibile</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1073,22 +1073,22 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
+          <t>Disponibile</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Scorta</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
           <t>Dell Latitude 7320 Detachable</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="F23" t="inlineStr">
         <is>
           <t>4HK210</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>Disponibile</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>Scorta</t>
         </is>
       </c>
     </row>
@@ -1112,20 +1112,20 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
+          <t>Disponibile</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="inlineStr">
+        <is>
           <t>Lenovo ThinkPad T14 Gen 5</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="F25" t="inlineStr">
         <is>
           <t>PF5DR01</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>Disponibile</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1140,22 +1140,22 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
+          <t>Disponibile</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Postazione 1</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
           <t>Lenovo ThinkPad T14 Gen 4</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="F26" t="inlineStr">
         <is>
           <t>PF4DR02</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>Disponibile</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>Postazione 1</t>
         </is>
       </c>
     </row>
@@ -1172,20 +1172,20 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
+          <t>Disponibile</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="inlineStr">
+        <is>
           <t>Lenovo ThinkPad T14 Gen 5</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="F27" t="inlineStr">
         <is>
           <t>PF5DR03</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>Disponibile</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1200,22 +1200,22 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
+          <t>In attesa ritiro</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Batteria da sostituire</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
           <t>Lenovo ThinkPad T14 Gen 4</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="F28" t="inlineStr">
         <is>
           <t>PF4DR04</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>In attesa ritiro</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>Batteria da sostituire</t>
         </is>
       </c>
     </row>
@@ -1232,20 +1232,20 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
+          <t>Guasto in attesa tecnico</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr"/>
+      <c r="E29" t="inlineStr">
+        <is>
           <t>Lenovo ThinkPad T14 Gen 5</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="F29" t="inlineStr">
         <is>
           <t>PF5DR05</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>Guasto in attesa tecnico</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1260,22 +1260,22 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
+          <t>Da rebuildare</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Con custodia</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
           <t>Lenovo ThinkPad T14 Gen 4</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
+      <c r="F30" t="inlineStr">
         <is>
           <t>PF4DR06</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>Da rebuildare</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>Con custodia</t>
         </is>
       </c>
     </row>
@@ -1292,20 +1292,20 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
+          <t>Controllare</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="inlineStr">
+        <is>
           <t>Lenovo ThinkPad T14 Gen 5</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="F31" t="inlineStr">
         <is>
           <t>PF5DR07</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>Controllare</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1320,22 +1320,22 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
+          <t>Disponibile</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>In verifica</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
           <t>Dell Latitude 7320 Detachable</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr">
+      <c r="F32" t="inlineStr">
         <is>
           <t>7HD308</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>Disponibile</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>In verifica</t>
         </is>
       </c>
     </row>
@@ -1352,20 +1352,20 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
+          <t>Disponibile</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr"/>
+      <c r="E33" t="inlineStr">
+        <is>
           <t>Dell Latitude 7230 Rugged Extreme</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
+      <c r="F33" t="inlineStr">
         <is>
           <t>8HD309</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>Disponibile</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1380,22 +1380,22 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
+          <t>Disponibile</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Scorta</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
           <t>Dell Latitude 7320 Detachable</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
+      <c r="F34" t="inlineStr">
         <is>
           <t>4HD310</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>Disponibile</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>Scorta</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Doppioni rifiutati, copia locale ricordata, Note prima di Stato
Un asset tag gia' presente non entra piu' in silenzio: il programma non
inserisce niente e dice dove sta il dispositivo che ce l'ha gia', con
modello e stanza, cosi' si capisce subito se e' un errore di battitura o
un dispositivo gia' registrato.

Ogni cinque record toccati - aggiunti, modificati o eliminati, contati
per record e non per operazione - il programma ricorda di portarsi via
una copia locale. Le copie automatiche stanno sulla share accanto ai
dati: coprono l'errore umano, non la cartella che sparisce, e quella
copia la deve volere qualcuno.

Note passa prima di Stato nell'elenco, nel modello da compilare e nei
file di prova; l'esportazione scende a tre campi.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Collaudo/Inventario_di_prova.xlsx
+++ b/Collaudo/Inventario_di_prova.xlsx
@@ -440,8 +440,8 @@
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="9" customWidth="1" min="2" max="2"/>
-    <col width="27" customWidth="1" min="3" max="3"/>
-    <col width="25" customWidth="1" min="4" max="4"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="27" customWidth="1" min="4" max="4"/>
     <col width="36" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
   </cols>
@@ -459,12 +459,12 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>Stato</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Note</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -496,12 +496,12 @@
           <t>Laptop</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Disponibile</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr"/>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Disponibile</t>
+        </is>
+      </c>
       <c r="E3" t="inlineStr">
         <is>
           <t>Lenovo ThinkPad T14 Gen 5</t>
@@ -526,12 +526,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Disponibile</t>
+          <t>Postazione 1</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Postazione 1</t>
+          <t>Disponibile</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -556,12 +556,12 @@
           <t>Laptop</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Disponibile</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr"/>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Disponibile</t>
+        </is>
+      </c>
       <c r="E5" t="inlineStr">
         <is>
           <t>Lenovo ThinkPad T14 Gen 5</t>
@@ -586,12 +586,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
+          <t>Batteria da sostituire</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
           <t>In attesa ritiro</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Batteria da sostituire</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -616,12 +616,12 @@
           <t>Laptop</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr">
         <is>
           <t>Guasto in attesa tecnico</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
           <t>Lenovo ThinkPad T14 Gen 5</t>
@@ -646,12 +646,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
+          <t>Con custodia</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
           <t>Da rebuildare</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Con custodia</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -676,12 +676,12 @@
           <t>Laptop</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr">
         <is>
           <t>Controllare</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
           <t>Lenovo ThinkPad T14 Gen 5</t>
@@ -706,12 +706,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Disponibile</t>
+          <t>In verifica</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>In verifica</t>
+          <t>Disponibile</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -736,12 +736,12 @@
           <t>Tablet</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Disponibile</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr"/>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Disponibile</t>
+        </is>
+      </c>
       <c r="E11" t="inlineStr">
         <is>
           <t>Dell Latitude 7230 Rugged Extreme</t>
@@ -766,12 +766,12 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Disponibile</t>
+          <t>Scorta</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Scorta</t>
+          <t>Disponibile</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -803,12 +803,12 @@
           <t>Laptop</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Disponibile</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr"/>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Disponibile</t>
+        </is>
+      </c>
       <c r="E14" t="inlineStr">
         <is>
           <t>Lenovo ThinkPad T14 Gen 5</t>
@@ -833,12 +833,12 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Disponibile</t>
+          <t>Postazione 1</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Postazione 1</t>
+          <t>Disponibile</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -863,12 +863,12 @@
           <t>Laptop</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Disponibile</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr"/>
+      <c r="C16" t="inlineStr"/>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Disponibile</t>
+        </is>
+      </c>
       <c r="E16" t="inlineStr">
         <is>
           <t>Lenovo ThinkPad T14 Gen 5</t>
@@ -893,12 +893,12 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
+          <t>Batteria da sostituire</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
           <t>In attesa ritiro</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>Batteria da sostituire</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -923,12 +923,12 @@
           <t>Laptop</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C18" t="inlineStr"/>
+      <c r="D18" t="inlineStr">
         <is>
           <t>Guasto in attesa tecnico</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
           <t>Lenovo ThinkPad T14 Gen 5</t>
@@ -953,12 +953,12 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
+          <t>Con custodia</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
           <t>Da rebuildare</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>Con custodia</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -983,12 +983,12 @@
           <t>Laptop</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C20" t="inlineStr"/>
+      <c r="D20" t="inlineStr">
         <is>
           <t>Controllare</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
           <t>Lenovo ThinkPad T14 Gen 5</t>
@@ -1013,12 +1013,12 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Disponibile</t>
+          <t>In verifica</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>In verifica</t>
+          <t>Disponibile</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1043,12 +1043,12 @@
           <t>Tablet</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>Disponibile</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr"/>
+      <c r="C22" t="inlineStr"/>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Disponibile</t>
+        </is>
+      </c>
       <c r="E22" t="inlineStr">
         <is>
           <t>Dell Latitude 7230 Rugged Extreme</t>
@@ -1073,12 +1073,12 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Disponibile</t>
+          <t>Scorta</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Scorta</t>
+          <t>Disponibile</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1110,12 +1110,12 @@
           <t>Laptop</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>Disponibile</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr"/>
+      <c r="C25" t="inlineStr"/>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Disponibile</t>
+        </is>
+      </c>
       <c r="E25" t="inlineStr">
         <is>
           <t>Lenovo ThinkPad T14 Gen 5</t>
@@ -1140,12 +1140,12 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Disponibile</t>
+          <t>Postazione 1</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Postazione 1</t>
+          <t>Disponibile</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1170,12 +1170,12 @@
           <t>Laptop</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>Disponibile</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr"/>
+      <c r="C27" t="inlineStr"/>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Disponibile</t>
+        </is>
+      </c>
       <c r="E27" t="inlineStr">
         <is>
           <t>Lenovo ThinkPad T14 Gen 5</t>
@@ -1200,12 +1200,12 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
+          <t>Batteria da sostituire</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
           <t>In attesa ritiro</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>Batteria da sostituire</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -1230,12 +1230,12 @@
           <t>Laptop</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C29" t="inlineStr"/>
+      <c r="D29" t="inlineStr">
         <is>
           <t>Guasto in attesa tecnico</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
           <t>Lenovo ThinkPad T14 Gen 5</t>
@@ -1260,12 +1260,12 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
+          <t>Con custodia</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
           <t>Da rebuildare</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>Con custodia</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -1290,12 +1290,12 @@
           <t>Laptop</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C31" t="inlineStr"/>
+      <c r="D31" t="inlineStr">
         <is>
           <t>Controllare</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
           <t>Lenovo ThinkPad T14 Gen 5</t>
@@ -1320,12 +1320,12 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Disponibile</t>
+          <t>In verifica</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>In verifica</t>
+          <t>Disponibile</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -1350,12 +1350,12 @@
           <t>Tablet</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>Disponibile</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr"/>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Disponibile</t>
+        </is>
+      </c>
       <c r="E33" t="inlineStr">
         <is>
           <t>Dell Latitude 7230 Rugged Extreme</t>
@@ -1380,12 +1380,12 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Disponibile</t>
+          <t>Scorta</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Scorta</t>
+          <t>Disponibile</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">

</xml_diff>